<commit_message>
Fix test files with realistic ML patterns and resolve MLflow deprecation warning
</commit_message>
<xml_diff>
--- a/test files/bci_motor_imagery.xlsx
+++ b/test files/bci_motor_imagery.xlsx
@@ -489,19 +489,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.692258350163164</v>
+        <v>5.79802849180674</v>
       </c>
       <c r="E2" t="n">
-        <v>4.445256367183231</v>
+        <v>2.417041419297289</v>
       </c>
       <c r="F2" t="n">
-        <v>2.894212124407885</v>
+        <v>3.823844269050346</v>
       </c>
       <c r="G2" t="n">
-        <v>4.32850400884438</v>
+        <v>2.261514928204013</v>
       </c>
       <c r="H2" t="n">
-        <v>404.0019263429275</v>
+        <v>312.9753987582999</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
@@ -516,26 +516,26 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7.034650565248598</v>
+        <v>5.359517825830491</v>
       </c>
       <c r="E3" t="n">
-        <v>4.508095216433742</v>
+        <v>2.667424775320082</v>
       </c>
       <c r="F3" t="n">
-        <v>4.630923137623631</v>
+        <v>4.005257642403263</v>
       </c>
       <c r="G3" t="n">
-        <v>1.963663711064272</v>
+        <v>1.209560932988242</v>
       </c>
       <c r="H3" t="n">
-        <v>312.8561278710915</v>
+        <v>304.2449057846555</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -547,23 +547,23 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2.668886003045618</v>
+        <v>2.64517736293962</v>
       </c>
       <c r="E4" t="n">
-        <v>5.261982020958452</v>
+        <v>4.352031853205322</v>
       </c>
       <c r="F4" t="n">
-        <v>3.137325575855229</v>
+        <v>0.6375410837434836</v>
       </c>
       <c r="G4" t="n">
-        <v>1.94824956990775</v>
+        <v>3.218856235379514</v>
       </c>
       <c r="H4" t="n">
-        <v>339.7690432918933</v>
+        <v>289.6150663899673</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
@@ -578,23 +578,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7.182890740577721</v>
+        <v>2.688548399557164</v>
       </c>
       <c r="E5" t="n">
-        <v>3.682578781506479</v>
+        <v>5.077993718975556</v>
       </c>
       <c r="F5" t="n">
-        <v>4.408921560271723</v>
+        <v>0.4301896719618803</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7362713907035761</v>
+        <v>3.185262519537875</v>
       </c>
       <c r="H5" t="n">
-        <v>321.181129640311</v>
+        <v>337.9316140073782</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
@@ -609,23 +609,23 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6.636723638803254</v>
+        <v>1.727808637737409</v>
       </c>
       <c r="E6" t="n">
-        <v>2.834469894908653</v>
+        <v>2.055461294854933</v>
       </c>
       <c r="F6" t="n">
-        <v>5.002907340126667</v>
+        <v>0.7396025690310788</v>
       </c>
       <c r="G6" t="n">
-        <v>3.877082071242785</v>
+        <v>1.350279207338269</v>
       </c>
       <c r="H6" t="n">
-        <v>284.5472203851868</v>
+        <v>301.9808393024359</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
@@ -640,26 +640,26 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4.563894170293278</v>
+        <v>1.854153125103362</v>
       </c>
       <c r="E7" t="n">
-        <v>7.054527743540428</v>
+        <v>1.489223902662201</v>
       </c>
       <c r="F7" t="n">
-        <v>2.795780632175891</v>
+        <v>1.135297845440992</v>
       </c>
       <c r="G7" t="n">
-        <v>3.562484233629603</v>
+        <v>0.9865404784630052</v>
       </c>
       <c r="H7" t="n">
-        <v>347.5773448008769</v>
+        <v>319.8341641303962</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -671,26 +671,26 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4.026690500948473</v>
+        <v>5.075781438472232</v>
       </c>
       <c r="E8" t="n">
-        <v>7.193728562719391</v>
+        <v>3.645409445020285</v>
       </c>
       <c r="F8" t="n">
-        <v>3.351955365935016</v>
+        <v>3.125318157002853</v>
       </c>
       <c r="G8" t="n">
-        <v>3.723966519591114</v>
+        <v>1.824197925672135</v>
       </c>
       <c r="H8" t="n">
-        <v>332.583159351469</v>
+        <v>280.1544185330471</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -706,19 +706,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6.247741433217951</v>
+        <v>4.637802865108386</v>
       </c>
       <c r="E9" t="n">
-        <v>5.269373689194768</v>
+        <v>4.653046821237703</v>
       </c>
       <c r="F9" t="n">
-        <v>3.980004184566379</v>
+        <v>3.529056623369166</v>
       </c>
       <c r="G9" t="n">
-        <v>1.81698877594322</v>
+        <v>2.394548794280936</v>
       </c>
       <c r="H9" t="n">
-        <v>293.6248067344027</v>
+        <v>272.5011735938934</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
@@ -737,19 +737,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3.818389758656554</v>
+        <v>5.223616737424128</v>
       </c>
       <c r="E10" t="n">
-        <v>5.37823325850143</v>
+        <v>3.134273335731349</v>
       </c>
       <c r="F10" t="n">
-        <v>3.76750003902252</v>
+        <v>3.67180914478423</v>
       </c>
       <c r="G10" t="n">
-        <v>1.395751044080147</v>
+        <v>0.618479922318633</v>
       </c>
       <c r="H10" t="n">
-        <v>337.3276135142535</v>
+        <v>329.7225190818439</v>
       </c>
       <c r="I10" t="n">
         <v>1</v>
@@ -764,23 +764,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3.893003075080814</v>
+        <v>5.26895063175021</v>
       </c>
       <c r="E11" t="n">
-        <v>6.891520964870011</v>
+        <v>2.849273676827823</v>
       </c>
       <c r="F11" t="n">
-        <v>3.760490732920501</v>
+        <v>3.943874229796679</v>
       </c>
       <c r="G11" t="n">
-        <v>1.680381691566667</v>
+        <v>1.947166165054381</v>
       </c>
       <c r="H11" t="n">
-        <v>299.4275962347999</v>
+        <v>342.6499339173421</v>
       </c>
       <c r="I11" t="n">
         <v>1</v>
@@ -795,23 +795,23 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>4.964197393992907</v>
+        <v>1.996469486066417</v>
       </c>
       <c r="E12" t="n">
-        <v>5.23498033490561</v>
+        <v>5.314472574489272</v>
       </c>
       <c r="F12" t="n">
-        <v>1.666526172822265</v>
+        <v>1.665631715701782</v>
       </c>
       <c r="G12" t="n">
-        <v>2.077427727641296</v>
+        <v>3.98777256356118</v>
       </c>
       <c r="H12" t="n">
-        <v>275.8201855956588</v>
+        <v>305.6247728646413</v>
       </c>
       <c r="I12" t="n">
         <v>1</v>
@@ -826,26 +826,26 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1.804649606319623</v>
+        <v>2.38860461400171</v>
       </c>
       <c r="E13" t="n">
-        <v>4.371383141084531</v>
+        <v>6.207829806820421</v>
       </c>
       <c r="F13" t="n">
-        <v>2.151583271838201</v>
+        <v>1.050896030272161</v>
       </c>
       <c r="G13" t="n">
-        <v>4.553958908912854</v>
+        <v>3.917397709615214</v>
       </c>
       <c r="H13" t="n">
-        <v>271.7733098259151</v>
+        <v>328.8968415298691</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -857,23 +857,23 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2.825036602397441</v>
+        <v>2.180818012523817</v>
       </c>
       <c r="E14" t="n">
-        <v>5.059008690166195</v>
+        <v>1.677440122697438</v>
       </c>
       <c r="F14" t="n">
-        <v>2.504732979058812</v>
+        <v>1.344558242203366</v>
       </c>
       <c r="G14" t="n">
-        <v>4.000126723782502</v>
+        <v>1.815214626586388</v>
       </c>
       <c r="H14" t="n">
-        <v>330.8023448385192</v>
+        <v>318.9252188267014</v>
       </c>
       <c r="I14" t="n">
         <v>1</v>
@@ -888,23 +888,23 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4.526508126497776</v>
+        <v>2.782321827907003</v>
       </c>
       <c r="E15" t="n">
-        <v>7.089752955751209</v>
+        <v>1.800680804992399</v>
       </c>
       <c r="F15" t="n">
-        <v>4.214420803468676</v>
+        <v>1.175654365010101</v>
       </c>
       <c r="G15" t="n">
-        <v>2.54177935937968</v>
+        <v>0.6324998165634388</v>
       </c>
       <c r="H15" t="n">
-        <v>304.6907628028622</v>
+        <v>351.2747485201826</v>
       </c>
       <c r="I15" t="n">
         <v>1</v>
@@ -919,23 +919,23 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>5.713544048318899</v>
+        <v>4.346229678513741</v>
       </c>
       <c r="E16" t="n">
-        <v>5.079982502643209</v>
+        <v>4.749978800058223</v>
       </c>
       <c r="F16" t="n">
-        <v>1.764625092873114</v>
+        <v>3.88673642684491</v>
       </c>
       <c r="G16" t="n">
-        <v>3.299251993259985</v>
+        <v>2.689037869035812</v>
       </c>
       <c r="H16" t="n">
-        <v>380.0681607617585</v>
+        <v>295.7451919132044</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -954,22 +954,22 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.797639092881982</v>
+        <v>4.148770069490824</v>
       </c>
       <c r="E17" t="n">
-        <v>3.995926198019671</v>
+        <v>4.851013832067363</v>
       </c>
       <c r="F17" t="n">
-        <v>4.523226707178839</v>
+        <v>3.694911991759216</v>
       </c>
       <c r="G17" t="n">
-        <v>2.321637753852261</v>
+        <v>3.154270122033767</v>
       </c>
       <c r="H17" t="n">
-        <v>318.2816754664817</v>
+        <v>329.4353868758952</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -985,22 +985,22 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4.703584282967476</v>
+        <v>5.558246529608824</v>
       </c>
       <c r="E18" t="n">
-        <v>5.220503073927646</v>
+        <v>3.081186994319733</v>
       </c>
       <c r="F18" t="n">
-        <v>3.779834114078683</v>
+        <v>3.148973453061324</v>
       </c>
       <c r="G18" t="n">
-        <v>3.364279760781657</v>
+        <v>1.336168926701116</v>
       </c>
       <c r="H18" t="n">
-        <v>288.5918682618567</v>
+        <v>308.2367554060353</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1012,26 +1012,26 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2.579810887793552</v>
+        <v>4.621891031120729</v>
       </c>
       <c r="E19" t="n">
-        <v>5.984334706303646</v>
+        <v>0.906894371461918</v>
       </c>
       <c r="F19" t="n">
-        <v>4.154230224722774</v>
+        <v>3.672758971944383</v>
       </c>
       <c r="G19" t="n">
-        <v>1.861904262258002</v>
+        <v>1.302241774209853</v>
       </c>
       <c r="H19" t="n">
-        <v>326.3127055457565</v>
+        <v>311.3258943059017</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1043,26 +1043,26 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>6.39872577840548</v>
+        <v>2.403228573000395</v>
       </c>
       <c r="E20" t="n">
-        <v>5.804380242358548</v>
+        <v>5.742430514088723</v>
       </c>
       <c r="F20" t="n">
-        <v>2.070466922755001</v>
+        <v>2.443092950605265</v>
       </c>
       <c r="G20" t="n">
-        <v>3.750251445973931</v>
+        <v>3.58728890641592</v>
       </c>
       <c r="H20" t="n">
-        <v>268.2293071370157</v>
+        <v>327.7265117216829</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1074,23 +1074,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>5.330123494341472</v>
+        <v>2.4553324505403</v>
       </c>
       <c r="E21" t="n">
-        <v>5.829235922107414</v>
+        <v>5.488869517293016</v>
       </c>
       <c r="F21" t="n">
-        <v>3.07230236269013</v>
+        <v>0.6632476890048884</v>
       </c>
       <c r="G21" t="n">
-        <v>2.150296702415607</v>
+        <v>2.963734082782171</v>
       </c>
       <c r="H21" t="n">
-        <v>316.6347503790119</v>
+        <v>290.2224146179043</v>
       </c>
       <c r="I21" t="n">
         <v>1</v>
@@ -1105,26 +1105,26 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5.462818853958826</v>
+        <v>2.030115104970513</v>
       </c>
       <c r="E22" t="n">
-        <v>3.759983481299855</v>
+        <v>3.231621056242643</v>
       </c>
       <c r="F22" t="n">
-        <v>3.298942786131316</v>
+        <v>1.123055614087551</v>
       </c>
       <c r="G22" t="n">
-        <v>3.805915028543157</v>
+        <v>1.320618936933445</v>
       </c>
       <c r="H22" t="n">
-        <v>332.766671059131</v>
+        <v>318.9586469088427</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1136,23 +1136,23 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>5.732375926977342</v>
+        <v>1.415660981190234</v>
       </c>
       <c r="E23" t="n">
-        <v>6.155155349837685</v>
+        <v>2.383648419353202</v>
       </c>
       <c r="F23" t="n">
-        <v>3.254967002022694</v>
+        <v>0.7400829690022566</v>
       </c>
       <c r="G23" t="n">
-        <v>2.572577091805658</v>
+        <v>0.8898655576172223</v>
       </c>
       <c r="H23" t="n">
-        <v>327.8268923054122</v>
+        <v>343.1942256766775</v>
       </c>
       <c r="I23" t="n">
         <v>1</v>
@@ -1167,23 +1167,23 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>5.117191255242179</v>
+        <v>5.48195601765527</v>
       </c>
       <c r="E24" t="n">
-        <v>5.042698908818434</v>
+        <v>3.518704256045404</v>
       </c>
       <c r="F24" t="n">
-        <v>3.295657400846717</v>
+        <v>3.352114256280162</v>
       </c>
       <c r="G24" t="n">
-        <v>2.209924046401726</v>
+        <v>4.314273375485987</v>
       </c>
       <c r="H24" t="n">
-        <v>372.1119972207903</v>
+        <v>290.2839102460794</v>
       </c>
       <c r="I24" t="n">
         <v>1</v>
@@ -1202,19 +1202,19 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4.274340862139002</v>
+        <v>4.10359158927806</v>
       </c>
       <c r="E25" t="n">
-        <v>3.932313248795817</v>
+        <v>5.694623467574923</v>
       </c>
       <c r="F25" t="n">
-        <v>2.723473519604888</v>
+        <v>3.524153649381228</v>
       </c>
       <c r="G25" t="n">
-        <v>4.612996717249656</v>
+        <v>3.005486607444082</v>
       </c>
       <c r="H25" t="n">
-        <v>423.900685033778</v>
+        <v>309.0338210950237</v>
       </c>
       <c r="I25" t="n">
         <v>1</v>
@@ -1233,22 +1233,22 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>6.694481823080462</v>
+        <v>4.862617771764337</v>
       </c>
       <c r="E26" t="n">
-        <v>6.14322757047805</v>
+        <v>2.784155458381109</v>
       </c>
       <c r="F26" t="n">
-        <v>3.135207081063659</v>
+        <v>3.040287882883098</v>
       </c>
       <c r="G26" t="n">
-        <v>3.176946184893766</v>
+        <v>2.27496720250877</v>
       </c>
       <c r="H26" t="n">
-        <v>346.8558948536514</v>
+        <v>296.5024012299129</v>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1260,23 +1260,23 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>5.235321721641159</v>
+        <v>5.306763090276594</v>
       </c>
       <c r="E27" t="n">
-        <v>4.319541726624854</v>
+        <v>2.285952984539084</v>
       </c>
       <c r="F27" t="n">
-        <v>4.033563955065187</v>
+        <v>3.778060899266983</v>
       </c>
       <c r="G27" t="n">
-        <v>2.677818628951443</v>
+        <v>2.021930305459329</v>
       </c>
       <c r="H27" t="n">
-        <v>367.1518531114208</v>
+        <v>335.7934448400409</v>
       </c>
       <c r="I27" t="n">
         <v>1</v>
@@ -1291,23 +1291,23 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4.751420856989863</v>
+        <v>1.535510059263264</v>
       </c>
       <c r="E28" t="n">
-        <v>2.63855397716667</v>
+        <v>5.610780315119382</v>
       </c>
       <c r="F28" t="n">
-        <v>1.83348769155911</v>
+        <v>1.629941397124212</v>
       </c>
       <c r="G28" t="n">
-        <v>3.758178308351264</v>
+        <v>3.890911435888655</v>
       </c>
       <c r="H28" t="n">
-        <v>421.7385063862896</v>
+        <v>282.8914786736576</v>
       </c>
       <c r="I28" t="n">
         <v>1</v>
@@ -1322,23 +1322,23 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>4.987018019119244</v>
+        <v>1.707726032149434</v>
       </c>
       <c r="E29" t="n">
-        <v>3.499096428334517</v>
+        <v>5.870584507306687</v>
       </c>
       <c r="F29" t="n">
-        <v>4.547050118905403</v>
+        <v>2.108535398490055</v>
       </c>
       <c r="G29" t="n">
-        <v>1.660008930425115</v>
+        <v>3.613144134749438</v>
       </c>
       <c r="H29" t="n">
-        <v>279.750966087341</v>
+        <v>345.4220429772992</v>
       </c>
       <c r="I29" t="n">
         <v>1</v>
@@ -1353,23 +1353,23 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>4.95505240026689</v>
+        <v>2.146536236649341</v>
       </c>
       <c r="E30" t="n">
-        <v>4.727544600429376</v>
+        <v>1.642824290986816</v>
       </c>
       <c r="F30" t="n">
-        <v>3.981898956368448</v>
+        <v>1.946309804457903</v>
       </c>
       <c r="G30" t="n">
-        <v>4.106863589260358</v>
+        <v>1.389533168364715</v>
       </c>
       <c r="H30" t="n">
-        <v>325.2250963510003</v>
+        <v>284.2608950839206</v>
       </c>
       <c r="I30" t="n">
         <v>1</v>
@@ -1384,23 +1384,23 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>4.736351594112032</v>
+        <v>2.328276804316915</v>
       </c>
       <c r="E31" t="n">
-        <v>5.867453423166919</v>
+        <v>1.624410287668036</v>
       </c>
       <c r="F31" t="n">
-        <v>2.034798107316667</v>
+        <v>0.7478287787517879</v>
       </c>
       <c r="G31" t="n">
-        <v>2.860555293591551</v>
+        <v>1.507990943972317</v>
       </c>
       <c r="H31" t="n">
-        <v>300.8801387165337</v>
+        <v>358.0516856721171</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -1415,26 +1415,26 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>5.669159543761861</v>
+        <v>5.075442111996143</v>
       </c>
       <c r="E32" t="n">
-        <v>3.703895071867863</v>
+        <v>5.827755087857764</v>
       </c>
       <c r="F32" t="n">
-        <v>3.383836043455322</v>
+        <v>2.852767130398278</v>
       </c>
       <c r="G32" t="n">
-        <v>3.600787715668437</v>
+        <v>2.547758301385506</v>
       </c>
       <c r="H32" t="n">
-        <v>353.7063084104429</v>
+        <v>293.3145671112343</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -1450,19 +1450,19 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3.596209666816447</v>
+        <v>3.928932800524193</v>
       </c>
       <c r="E33" t="n">
-        <v>4.639006309343698</v>
+        <v>5.115071483733627</v>
       </c>
       <c r="F33" t="n">
-        <v>3.901498776158045</v>
+        <v>2.856243295083714</v>
       </c>
       <c r="G33" t="n">
-        <v>1.452126538976914</v>
+        <v>3.72562918241198</v>
       </c>
       <c r="H33" t="n">
-        <v>330.8647567790648</v>
+        <v>336.1388001107599</v>
       </c>
       <c r="I33" t="n">
         <v>1</v>
@@ -1481,22 +1481,22 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>3.705813446389538</v>
+        <v>5.341205900057227</v>
       </c>
       <c r="E34" t="n">
-        <v>3.175089152505413</v>
+        <v>4.132101499953771</v>
       </c>
       <c r="F34" t="n">
-        <v>1.764706676114316</v>
+        <v>3.812833673882503</v>
       </c>
       <c r="G34" t="n">
-        <v>2.617574041867004</v>
+        <v>1.071421221791859</v>
       </c>
       <c r="H34" t="n">
-        <v>287.2627072038426</v>
+        <v>287.8732250581666</v>
       </c>
       <c r="I34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1508,23 +1508,23 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5.838895534142953</v>
+        <v>5.789483449145911</v>
       </c>
       <c r="E35" t="n">
-        <v>6.473049374359716</v>
+        <v>2.425520566671004</v>
       </c>
       <c r="F35" t="n">
-        <v>3.041978433376601</v>
+        <v>3.870170408973869</v>
       </c>
       <c r="G35" t="n">
-        <v>3.004580139345484</v>
+        <v>1.273768883827665</v>
       </c>
       <c r="H35" t="n">
-        <v>320.4379126538818</v>
+        <v>343.3114938471082</v>
       </c>
       <c r="I35" t="n">
         <v>1</v>
@@ -1539,26 +1539,26 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>4.782140988908306</v>
+        <v>2.232091028759787</v>
       </c>
       <c r="E36" t="n">
-        <v>7.575996670933328</v>
+        <v>6.013839276594084</v>
       </c>
       <c r="F36" t="n">
-        <v>2.921484699164994</v>
+        <v>1.607046872065102</v>
       </c>
       <c r="G36" t="n">
-        <v>4.030299213618528</v>
+        <v>2.877130610644006</v>
       </c>
       <c r="H36" t="n">
-        <v>361.8769095862354</v>
+        <v>325.1954277755354</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -1570,23 +1570,23 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>6.457089653214644</v>
+        <v>2.731190427837302</v>
       </c>
       <c r="E37" t="n">
-        <v>7.413923786732481</v>
+        <v>5.638572233767079</v>
       </c>
       <c r="F37" t="n">
-        <v>2.354419457493106</v>
+        <v>1.095531554304819</v>
       </c>
       <c r="G37" t="n">
-        <v>3.680411063937483</v>
+        <v>4.028711754431188</v>
       </c>
       <c r="H37" t="n">
-        <v>267.8510147589973</v>
+        <v>321.5408257843891</v>
       </c>
       <c r="I37" t="n">
         <v>1</v>
@@ -1601,23 +1601,23 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>5.613318500947796</v>
+        <v>2.541525621587638</v>
       </c>
       <c r="E38" t="n">
-        <v>6.447469325729207</v>
+        <v>2.526901026017451</v>
       </c>
       <c r="F38" t="n">
-        <v>3.092356836764013</v>
+        <v>0.6489322528171635</v>
       </c>
       <c r="G38" t="n">
-        <v>2.607522962382583</v>
+        <v>0.8248699840339508</v>
       </c>
       <c r="H38" t="n">
-        <v>288.1062177744408</v>
+        <v>335.4510580162598</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
@@ -1632,23 +1632,23 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>4.171058134885651</v>
+        <v>2.256892975456104</v>
       </c>
       <c r="E39" t="n">
-        <v>6.293764935680392</v>
+        <v>2.011965907232919</v>
       </c>
       <c r="F39" t="n">
-        <v>2.39971342403721</v>
+        <v>1.548765595524957</v>
       </c>
       <c r="G39" t="n">
-        <v>3.317947757323382</v>
+        <v>1.774942531333411</v>
       </c>
       <c r="H39" t="n">
-        <v>282.1089965983276</v>
+        <v>320.219191182219</v>
       </c>
       <c r="I39" t="n">
         <v>1</v>
@@ -1663,23 +1663,23 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>5.862644544693012</v>
+        <v>5.167801234445242</v>
       </c>
       <c r="E40" t="n">
-        <v>1.892180713395196</v>
+        <v>4.955973875914059</v>
       </c>
       <c r="F40" t="n">
-        <v>4.374307068970737</v>
+        <v>2.810838453215793</v>
       </c>
       <c r="G40" t="n">
-        <v>4.256569101726981</v>
+        <v>3.45538153229596</v>
       </c>
       <c r="H40" t="n">
-        <v>333.0558622194764</v>
+        <v>296.8152435638729</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
@@ -1698,19 +1698,19 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>6.795786436938403</v>
+        <v>4.334226975281994</v>
       </c>
       <c r="E41" t="n">
-        <v>5.265759848330158</v>
+        <v>4.472254700572266</v>
       </c>
       <c r="F41" t="n">
-        <v>2.37335567867259</v>
+        <v>2.679202354889962</v>
       </c>
       <c r="G41" t="n">
-        <v>2.80001151657744</v>
+        <v>1.926902097011702</v>
       </c>
       <c r="H41" t="n">
-        <v>369.6206431845984</v>
+        <v>330.719136258099</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
@@ -1729,22 +1729,22 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>5.670469334181881</v>
+        <v>5.21684088052634</v>
       </c>
       <c r="E42" t="n">
-        <v>4.255861064510138</v>
+        <v>3.15337035818042</v>
       </c>
       <c r="F42" t="n">
-        <v>3.791978940013158</v>
+        <v>3.532140009547732</v>
       </c>
       <c r="G42" t="n">
-        <v>2.691135039564692</v>
+        <v>0.9611276110353469</v>
       </c>
       <c r="H42" t="n">
-        <v>239.6106213877596</v>
+        <v>298.540888722201</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -1756,26 +1756,26 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>5.998377414600195</v>
+        <v>5.907758649360805</v>
       </c>
       <c r="E43" t="n">
-        <v>6.320699541567351</v>
+        <v>3.933421574435477</v>
       </c>
       <c r="F43" t="n">
-        <v>1.344613612379836</v>
+        <v>4.421706879160267</v>
       </c>
       <c r="G43" t="n">
-        <v>1.110295357247087</v>
+        <v>2.181717745475852</v>
       </c>
       <c r="H43" t="n">
-        <v>323.7759425391433</v>
+        <v>344.8629793281463</v>
       </c>
       <c r="I43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -1787,23 +1787,23 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>4.742343724094895</v>
+        <v>1.284914448005436</v>
       </c>
       <c r="E44" t="n">
-        <v>1.193603186478007</v>
+        <v>5.611872588861656</v>
       </c>
       <c r="F44" t="n">
-        <v>2.838190196150039</v>
+        <v>1.169106767615806</v>
       </c>
       <c r="G44" t="n">
-        <v>2.72092766465719</v>
+        <v>3.926216667398112</v>
       </c>
       <c r="H44" t="n">
-        <v>283.0311713089926</v>
+        <v>296.224377847019</v>
       </c>
       <c r="I44" t="n">
         <v>1</v>
@@ -1818,23 +1818,23 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>6.489559824320754</v>
+        <v>2.431158135119861</v>
       </c>
       <c r="E45" t="n">
-        <v>5.289451554155267</v>
+        <v>5.036908553345947</v>
       </c>
       <c r="F45" t="n">
-        <v>3.012311157351359</v>
+        <v>2.330650865304077</v>
       </c>
       <c r="G45" t="n">
-        <v>1.260372961315478</v>
+        <v>3.332876454424816</v>
       </c>
       <c r="H45" t="n">
-        <v>360.2161109931994</v>
+        <v>310.4645928046825</v>
       </c>
       <c r="I45" t="n">
         <v>1</v>
@@ -1849,26 +1849,26 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4.128964377605534</v>
+        <v>2.882727120140548</v>
       </c>
       <c r="E46" t="n">
-        <v>4.678334324251396</v>
+        <v>2.202490855480478</v>
       </c>
       <c r="F46" t="n">
-        <v>2.805708949384469</v>
+        <v>0.6956464182659818</v>
       </c>
       <c r="G46" t="n">
-        <v>2.885665320966793</v>
+        <v>1.56714477882191</v>
       </c>
       <c r="H46" t="n">
-        <v>310.5212689771498</v>
+        <v>383.664685910379</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1880,23 +1880,23 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>5.507814538610775</v>
+        <v>2.516232630275574</v>
       </c>
       <c r="E47" t="n">
-        <v>6.677644899397107</v>
+        <v>1.634629298385173</v>
       </c>
       <c r="F47" t="n">
-        <v>2.603681702804609</v>
+        <v>0.6880321066947479</v>
       </c>
       <c r="G47" t="n">
-        <v>3.988135143242747</v>
+        <v>1.105043215517332</v>
       </c>
       <c r="H47" t="n">
-        <v>325.2269575630959</v>
+        <v>376.1601704141691</v>
       </c>
       <c r="I47" t="n">
         <v>1</v>
@@ -1911,23 +1911,23 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>8.854259228653898</v>
+        <v>2.231112861951649</v>
       </c>
       <c r="E48" t="n">
-        <v>7.321980580512108</v>
+        <v>3.782928651065997</v>
       </c>
       <c r="F48" t="n">
-        <v>2.332484974654878</v>
+        <v>2.848459109164104</v>
       </c>
       <c r="G48" t="n">
-        <v>0.8803605249531845</v>
+        <v>2.25133009082109</v>
       </c>
       <c r="H48" t="n">
-        <v>319.9465201919176</v>
+        <v>368.972339117949</v>
       </c>
       <c r="I48" t="n">
         <v>1</v>
@@ -1946,19 +1946,19 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>5.80832158403849</v>
+        <v>3.498901035427557</v>
       </c>
       <c r="E49" t="n">
-        <v>3.606730974480848</v>
+        <v>4.410111497422204</v>
       </c>
       <c r="F49" t="n">
-        <v>3.754540780014903</v>
+        <v>2.720601137247272</v>
       </c>
       <c r="G49" t="n">
-        <v>4.23420882462079</v>
+        <v>3.035105341384106</v>
       </c>
       <c r="H49" t="n">
-        <v>364.9687521275938</v>
+        <v>390.4399078535097</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -1977,22 +1977,22 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>4.368933154112197</v>
+        <v>4.91109480937123</v>
       </c>
       <c r="E50" t="n">
-        <v>3.674434346154777</v>
+        <v>2.777262084557962</v>
       </c>
       <c r="F50" t="n">
-        <v>3.99945785509538</v>
+        <v>3.599529847786735</v>
       </c>
       <c r="G50" t="n">
-        <v>2.669776873343801</v>
+        <v>1.199891561420603</v>
       </c>
       <c r="H50" t="n">
-        <v>401.9452612319113</v>
+        <v>322.0940625497006</v>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -2004,23 +2004,23 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>4.365061637462901</v>
+        <v>5.268811841882944</v>
       </c>
       <c r="E51" t="n">
-        <v>5.34574493181757</v>
+        <v>1.361573810506805</v>
       </c>
       <c r="F51" t="n">
-        <v>2.91783911414335</v>
+        <v>4.140270380838732</v>
       </c>
       <c r="G51" t="n">
-        <v>2.972835132873394</v>
+        <v>1.192433161114335</v>
       </c>
       <c r="H51" t="n">
-        <v>274.6133868047423</v>
+        <v>383.3395292484876</v>
       </c>
       <c r="I51" t="n">
         <v>1</v>
@@ -2035,26 +2035,26 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>4.892987454064484</v>
+        <v>2.40892894297865</v>
       </c>
       <c r="E52" t="n">
-        <v>7.600644037282312</v>
+        <v>5.852990323890745</v>
       </c>
       <c r="F52" t="n">
-        <v>1.90336249197836</v>
+        <v>1.640495933867516</v>
       </c>
       <c r="G52" t="n">
-        <v>2.497580219861458</v>
+        <v>3.188650240089703</v>
       </c>
       <c r="H52" t="n">
-        <v>281.8977552802139</v>
+        <v>313.7563324892818</v>
       </c>
       <c r="I52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -2066,26 +2066,26 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>6.276868672594116</v>
+        <v>2.2041994392047</v>
       </c>
       <c r="E53" t="n">
-        <v>5.090217015924524</v>
+        <v>5.126657701056232</v>
       </c>
       <c r="F53" t="n">
-        <v>4.793949331386828</v>
+        <v>1.32225567954182</v>
       </c>
       <c r="G53" t="n">
-        <v>1.286763117451341</v>
+        <v>3.976005546923347</v>
       </c>
       <c r="H53" t="n">
-        <v>332.8599161021883</v>
+        <v>363.5765074238711</v>
       </c>
       <c r="I53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -2097,26 +2097,26 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>5.218666263751073</v>
+        <v>2.40643105941948</v>
       </c>
       <c r="E54" t="n">
-        <v>3.081257876968504</v>
+        <v>2.314814420961806</v>
       </c>
       <c r="F54" t="n">
-        <v>2.120202567092119</v>
+        <v>0.868401995631171</v>
       </c>
       <c r="G54" t="n">
-        <v>2.21701082570376</v>
+        <v>0.9759275839212121</v>
       </c>
       <c r="H54" t="n">
-        <v>287.3439060679232</v>
+        <v>342.4188081536979</v>
       </c>
       <c r="I54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -2128,26 +2128,26 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>4.027208280142405</v>
+        <v>2.305185132716733</v>
       </c>
       <c r="E55" t="n">
-        <v>4.091197330755061</v>
+        <v>1.106164194034109</v>
       </c>
       <c r="F55" t="n">
-        <v>1.540577741516853</v>
+        <v>0.7117719582872581</v>
       </c>
       <c r="G55" t="n">
-        <v>5.097410068449484</v>
+        <v>0.9323189087275148</v>
       </c>
       <c r="H55" t="n">
-        <v>357.343350816011</v>
+        <v>354.8581195324032</v>
       </c>
       <c r="I55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -2159,23 +2159,23 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>4.024554510816965</v>
+        <v>4.347623157740946</v>
       </c>
       <c r="E56" t="n">
-        <v>5.303996246695192</v>
+        <v>5.269143796391033</v>
       </c>
       <c r="F56" t="n">
-        <v>0.9873780834802299</v>
+        <v>3.495249809392818</v>
       </c>
       <c r="G56" t="n">
-        <v>1.903954503746548</v>
+        <v>3.488105781600383</v>
       </c>
       <c r="H56" t="n">
-        <v>363.7646983633735</v>
+        <v>359.1643642146299</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
@@ -2194,22 +2194,22 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>5.22807399653447</v>
+        <v>4.514702689142931</v>
       </c>
       <c r="E57" t="n">
-        <v>5.360303642845935</v>
+        <v>4.332542641491171</v>
       </c>
       <c r="F57" t="n">
-        <v>3.09945189691266</v>
+        <v>3.512384826640714</v>
       </c>
       <c r="G57" t="n">
-        <v>1.41145763827445</v>
+        <v>2.837375722626875</v>
       </c>
       <c r="H57" t="n">
-        <v>298.1369475101417</v>
+        <v>301.6071595127486</v>
       </c>
       <c r="I57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -2225,19 +2225,19 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>5.063592480108186</v>
+        <v>5.558197578995631</v>
       </c>
       <c r="E58" t="n">
-        <v>3.94386854661144</v>
+        <v>2.857094215262148</v>
       </c>
       <c r="F58" t="n">
-        <v>2.782583614484764</v>
+        <v>3.090889658383264</v>
       </c>
       <c r="G58" t="n">
-        <v>3.141291027407103</v>
+        <v>2.54619363784273</v>
       </c>
       <c r="H58" t="n">
-        <v>289.458509334341</v>
+        <v>289.8194785550089</v>
       </c>
       <c r="I58" t="n">
         <v>1</v>
@@ -2252,23 +2252,23 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>5.682464253678532</v>
+        <v>4.77148683232736</v>
       </c>
       <c r="E59" t="n">
-        <v>4.061313959330567</v>
+        <v>2.962406997713867</v>
       </c>
       <c r="F59" t="n">
-        <v>4.030956649146339</v>
+        <v>3.833528051734896</v>
       </c>
       <c r="G59" t="n">
-        <v>2.914223484827684</v>
+        <v>1.150426710954041</v>
       </c>
       <c r="H59" t="n">
-        <v>309.0088391338912</v>
+        <v>319.7354886126258</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
@@ -2283,23 +2283,23 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>6.376234843677342</v>
+        <v>3.08507184005065</v>
       </c>
       <c r="E60" t="n">
-        <v>3.527648008165403</v>
+        <v>5.411765571098717</v>
       </c>
       <c r="F60" t="n">
-        <v>3.611084563445547</v>
+        <v>1.087251401603744</v>
       </c>
       <c r="G60" t="n">
-        <v>2.676670209204352</v>
+        <v>3.339307079173503</v>
       </c>
       <c r="H60" t="n">
-        <v>324.1607285585208</v>
+        <v>332.3879436282687</v>
       </c>
       <c r="I60" t="n">
         <v>1</v>
@@ -2314,23 +2314,23 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>9.091039553614248</v>
+        <v>2.161765268317615</v>
       </c>
       <c r="E61" t="n">
-        <v>6.711756775780693</v>
+        <v>5.240017955858464</v>
       </c>
       <c r="F61" t="n">
-        <v>3.290201224585038</v>
+        <v>1.601911363763734</v>
       </c>
       <c r="G61" t="n">
-        <v>3.014447943352256</v>
+        <v>3.779554601307264</v>
       </c>
       <c r="H61" t="n">
-        <v>332.5934875958077</v>
+        <v>346.1762477429144</v>
       </c>
       <c r="I61" t="n">
         <v>1</v>
@@ -2345,23 +2345,23 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>2.806949724848599</v>
+        <v>1.275957829251338</v>
       </c>
       <c r="E62" t="n">
-        <v>3.747837231059916</v>
+        <v>1.296268112811722</v>
       </c>
       <c r="F62" t="n">
-        <v>2.72863280453725</v>
+        <v>0.9126223114990255</v>
       </c>
       <c r="G62" t="n">
-        <v>3.644202610696157</v>
+        <v>1.114621139315261</v>
       </c>
       <c r="H62" t="n">
-        <v>229.8873176380332</v>
+        <v>329.3272269679401</v>
       </c>
       <c r="I62" t="n">
         <v>1</v>
@@ -2376,23 +2376,23 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>6.030293190929662</v>
+        <v>2.737678108474776</v>
       </c>
       <c r="E63" t="n">
-        <v>4.302808694122574</v>
+        <v>1.848837878961846</v>
       </c>
       <c r="F63" t="n">
-        <v>4.109977272197667</v>
+        <v>1.198174868403882</v>
       </c>
       <c r="G63" t="n">
-        <v>2.412836400214686</v>
+        <v>0.9270629595519384</v>
       </c>
       <c r="H63" t="n">
-        <v>281.3017792459952</v>
+        <v>318.5541354339256</v>
       </c>
       <c r="I63" t="n">
         <v>1</v>
@@ -2407,23 +2407,23 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5.147461562582436</v>
+        <v>4.725902992236662</v>
       </c>
       <c r="E64" t="n">
-        <v>4.260120625214071</v>
+        <v>3.920938339513374</v>
       </c>
       <c r="F64" t="n">
-        <v>4.867389901752532</v>
+        <v>3.311607908544703</v>
       </c>
       <c r="G64" t="n">
-        <v>3.194410208282617</v>
+        <v>3.919643347801546</v>
       </c>
       <c r="H64" t="n">
-        <v>303.8360260451767</v>
+        <v>316.7371955462943</v>
       </c>
       <c r="I64" t="n">
         <v>1</v>
@@ -2442,22 +2442,22 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>2.233135653334117</v>
+        <v>4.781198205469259</v>
       </c>
       <c r="E65" t="n">
-        <v>2.591064128726913</v>
+        <v>4.259759134358182</v>
       </c>
       <c r="F65" t="n">
-        <v>4.008979199129904</v>
+        <v>3.274605872657304</v>
       </c>
       <c r="G65" t="n">
-        <v>4.023874662130003</v>
+        <v>3.041791598711328</v>
       </c>
       <c r="H65" t="n">
-        <v>288.1204267301245</v>
+        <v>349.505129190754</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -2473,22 +2473,22 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>6.874296085477591</v>
+        <v>5.558605659129299</v>
       </c>
       <c r="E66" t="n">
-        <v>3.704877042773276</v>
+        <v>2.03619412968672</v>
       </c>
       <c r="F66" t="n">
-        <v>2.53646836915079</v>
+        <v>3.512255087129471</v>
       </c>
       <c r="G66" t="n">
-        <v>2.004711333245205</v>
+        <v>1.748999145622725</v>
       </c>
       <c r="H66" t="n">
-        <v>205.4116043058819</v>
+        <v>363.5343082338512</v>
       </c>
       <c r="I66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -2500,26 +2500,26 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>5.631759839872921</v>
+        <v>6.075562495651124</v>
       </c>
       <c r="E67" t="n">
-        <v>6.842206398929807</v>
+        <v>3.220246929048039</v>
       </c>
       <c r="F67" t="n">
-        <v>3.781565553882175</v>
+        <v>4.408043895121907</v>
       </c>
       <c r="G67" t="n">
-        <v>0.6778186560613708</v>
+        <v>1.444534032185245</v>
       </c>
       <c r="H67" t="n">
-        <v>244.4651013858123</v>
+        <v>349.2892737944331</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -2531,26 +2531,26 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>6.199709439230235</v>
+        <v>1.996166894691534</v>
       </c>
       <c r="E68" t="n">
-        <v>3.186068237313908</v>
+        <v>5.140364412733587</v>
       </c>
       <c r="F68" t="n">
-        <v>2.597910274532785</v>
+        <v>0.4380521378450966</v>
       </c>
       <c r="G68" t="n">
-        <v>3.670808492095916</v>
+        <v>3.237122489159619</v>
       </c>
       <c r="H68" t="n">
-        <v>267.7856589766253</v>
+        <v>297.2260201533891</v>
       </c>
       <c r="I68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -2562,23 +2562,23 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>2.450871582353476</v>
+        <v>2.590236271885725</v>
       </c>
       <c r="E69" t="n">
-        <v>3.554536547260449</v>
+        <v>4.352376089761469</v>
       </c>
       <c r="F69" t="n">
-        <v>1.894932684140026</v>
+        <v>1.681238229402651</v>
       </c>
       <c r="G69" t="n">
-        <v>5.502962575602973</v>
+        <v>3.785673755163394</v>
       </c>
       <c r="H69" t="n">
-        <v>315.3886319658712</v>
+        <v>349.1157146003963</v>
       </c>
       <c r="I69" t="n">
         <v>1</v>
@@ -2593,26 +2593,26 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4.669374608752687</v>
+        <v>1.339883396489679</v>
       </c>
       <c r="E70" t="n">
-        <v>3.001181339331111</v>
+        <v>2.915729382927177</v>
       </c>
       <c r="F70" t="n">
-        <v>2.100960937878055</v>
+        <v>1.671776048288515</v>
       </c>
       <c r="G70" t="n">
-        <v>2.992645346351185</v>
+        <v>1.012329739158118</v>
       </c>
       <c r="H70" t="n">
-        <v>302.5519122607476</v>
+        <v>268.6059641272737</v>
       </c>
       <c r="I70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -2624,26 +2624,26 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3.381204582658556</v>
+        <v>2.676936187082706</v>
       </c>
       <c r="E71" t="n">
-        <v>4.864082659653109</v>
+        <v>2.137817578943704</v>
       </c>
       <c r="F71" t="n">
-        <v>2.641821595862254</v>
+        <v>1.311489213988264</v>
       </c>
       <c r="G71" t="n">
-        <v>3.201932201065956</v>
+        <v>0.2190941594737066</v>
       </c>
       <c r="H71" t="n">
-        <v>294.737236698857</v>
+        <v>292.96118544006</v>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -2655,23 +2655,23 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>8.244651414020918</v>
+        <v>4.503670589802728</v>
       </c>
       <c r="E72" t="n">
-        <v>7.828215081899435</v>
+        <v>4.532886415635319</v>
       </c>
       <c r="F72" t="n">
-        <v>3.103959678963544</v>
+        <v>2.729960717112454</v>
       </c>
       <c r="G72" t="n">
-        <v>2.704191566906009</v>
+        <v>3.373709959408499</v>
       </c>
       <c r="H72" t="n">
-        <v>351.8605984317136</v>
+        <v>287.9713871185222</v>
       </c>
       <c r="I72" t="n">
         <v>0</v>
@@ -2690,22 +2690,22 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>6.716825518616572</v>
+        <v>4.400334360485094</v>
       </c>
       <c r="E73" t="n">
-        <v>4.800958667709392</v>
+        <v>3.5419869191207</v>
       </c>
       <c r="F73" t="n">
-        <v>5.060581152575459</v>
+        <v>3.321295085985123</v>
       </c>
       <c r="G73" t="n">
-        <v>4.588060841510259</v>
+        <v>3.636268088466281</v>
       </c>
       <c r="H73" t="n">
-        <v>351.8453465969505</v>
+        <v>366.2411299075455</v>
       </c>
       <c r="I73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -2721,22 +2721,22 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>3.978548325071807</v>
+        <v>5.699388407187755</v>
       </c>
       <c r="E74" t="n">
-        <v>5.100143188031584</v>
+        <v>2.050908078066068</v>
       </c>
       <c r="F74" t="n">
-        <v>2.118310524388132</v>
+        <v>4.275575987761261</v>
       </c>
       <c r="G74" t="n">
-        <v>2.922243067055133</v>
+        <v>1.557837317146429</v>
       </c>
       <c r="H74" t="n">
-        <v>325.9967461392749</v>
+        <v>355.3789155219148</v>
       </c>
       <c r="I74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -2748,26 +2748,26 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Left_Hand</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2.695041648575597</v>
+        <v>5.540511088846065</v>
       </c>
       <c r="E75" t="n">
-        <v>3.806829146199517</v>
+        <v>3.115947907931247</v>
       </c>
       <c r="F75" t="n">
-        <v>4.323488489691329</v>
+        <v>3.583044066254076</v>
       </c>
       <c r="G75" t="n">
-        <v>2.813435839985065</v>
+        <v>0.9898083763689226</v>
       </c>
       <c r="H75" t="n">
-        <v>324.8048113087464</v>
+        <v>311.9271668621315</v>
       </c>
       <c r="I75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -2779,23 +2779,23 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>5.291082599575632</v>
+        <v>2.887225569751088</v>
       </c>
       <c r="E76" t="n">
-        <v>4.907572932811592</v>
+        <v>6.321178934519409</v>
       </c>
       <c r="F76" t="n">
-        <v>2.682740448307431</v>
+        <v>1.017538269709948</v>
       </c>
       <c r="G76" t="n">
-        <v>3.910863814269203</v>
+        <v>3.84302572999922</v>
       </c>
       <c r="H76" t="n">
-        <v>285.7335779626636</v>
+        <v>351.7527346054876</v>
       </c>
       <c r="I76" t="n">
         <v>1</v>
@@ -2810,23 +2810,23 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Tongue</t>
+          <t>Right_Hand</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>6.63863300344154</v>
+        <v>1.444756308146131</v>
       </c>
       <c r="E77" t="n">
-        <v>6.843575459521423</v>
+        <v>6.031638136147691</v>
       </c>
       <c r="F77" t="n">
-        <v>0.9836150125546563</v>
+        <v>1.431461089479074</v>
       </c>
       <c r="G77" t="n">
-        <v>2.515727037803178</v>
+        <v>3.600067209586711</v>
       </c>
       <c r="H77" t="n">
-        <v>290.5203067737389</v>
+        <v>254.8740251560877</v>
       </c>
       <c r="I77" t="n">
         <v>1</v>
@@ -2841,23 +2841,23 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Left_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>2.397419591846106</v>
+        <v>2.814307772785646</v>
       </c>
       <c r="E78" t="n">
-        <v>5.21436408145726</v>
+        <v>1.309949270892554</v>
       </c>
       <c r="F78" t="n">
-        <v>2.494273997069662</v>
+        <v>0.5186470242579381</v>
       </c>
       <c r="G78" t="n">
-        <v>1.715306298924146</v>
+        <v>1.177780920441353</v>
       </c>
       <c r="H78" t="n">
-        <v>251.6940246749913</v>
+        <v>331.5219634681792</v>
       </c>
       <c r="I78" t="n">
         <v>1</v>
@@ -2872,23 +2872,23 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Right_Hand</t>
+          <t>Feet</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>3.602337993510246</v>
+        <v>1.983652625952953</v>
       </c>
       <c r="E79" t="n">
-        <v>8.197655123093245</v>
+        <v>2.561338842399011</v>
       </c>
       <c r="F79" t="n">
-        <v>4.176696993167691</v>
+        <v>0.6235216958016004</v>
       </c>
       <c r="G79" t="n">
-        <v>3.882300379545694</v>
+        <v>1.150835477379418</v>
       </c>
       <c r="H79" t="n">
-        <v>309.9699427288668</v>
+        <v>317.7408903573463</v>
       </c>
       <c r="I79" t="n">
         <v>1</v>
@@ -2903,23 +2903,23 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>Tongue</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>3.341622936479062</v>
+        <v>4.756618772267794</v>
       </c>
       <c r="E80" t="n">
-        <v>6.889219568458537</v>
+        <v>3.842084149570852</v>
       </c>
       <c r="F80" t="n">
-        <v>3.344669519329236</v>
+        <v>2.691679849597984</v>
       </c>
       <c r="G80" t="n">
-        <v>2.408452792327854</v>
+        <v>2.364471886866629</v>
       </c>
       <c r="H80" t="n">
-        <v>351.4296515884479</v>
+        <v>318.1196270818048</v>
       </c>
       <c r="I80" t="n">
         <v>1</v>
@@ -2938,22 +2938,22 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>6.300419248865881</v>
+        <v>5.168599624350867</v>
       </c>
       <c r="E81" t="n">
-        <v>4.8705254818326</v>
+        <v>4.187321570516533</v>
       </c>
       <c r="F81" t="n">
-        <v>3.404451198663957</v>
+        <v>2.714597191218838</v>
       </c>
       <c r="G81" t="n">
-        <v>2.024539972323987</v>
+        <v>2.510700556026907</v>
       </c>
       <c r="H81" t="n">
-        <v>374.1731958709824</v>
+        <v>303.2292352029843</v>
       </c>
       <c r="I81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2967,7 +2967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2988,7 +2988,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Latency_ms</t>
+          <t>C3_beta_power</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>C4_beta_power</t>
         </is>
       </c>
     </row>
@@ -2999,13 +3004,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5.353475431375124</v>
+        <v>2.210155059501588</v>
       </c>
       <c r="C2" t="n">
-        <v>5.072372375529863</v>
+        <v>1.988610847425281</v>
       </c>
       <c r="D2" t="n">
-        <v>328.6202913334338</v>
+        <v>1.017508583872277</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.133725706675696</v>
       </c>
     </row>
     <row r="3">
@@ -3015,13 +3023,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4.664234580169353</v>
+        <v>5.381928985103188</v>
       </c>
       <c r="C3" t="n">
-        <v>4.379647222813923</v>
+        <v>2.707612558394596</v>
       </c>
       <c r="D3" t="n">
-        <v>303.4954366301412</v>
+        <v>3.758242721988251</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.514509478111504</v>
       </c>
     </row>
     <row r="4">
@@ -3031,13 +3042,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4.761671655835747</v>
+        <v>2.263915077613339</v>
       </c>
       <c r="C4" t="n">
-        <v>5.757368954071725</v>
+        <v>5.472158729246673</v>
       </c>
       <c r="D4" t="n">
-        <v>311.7258839433063</v>
+        <v>1.352580805070356</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3.563935486311542</v>
       </c>
     </row>
     <row r="5">
@@ -3047,13 +3061,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.385361882164007</v>
+        <v>4.461459953482079</v>
       </c>
       <c r="C5" t="n">
-        <v>4.830885880084379</v>
+        <v>4.47817674425835</v>
       </c>
       <c r="D5" t="n">
-        <v>325.115343007825</v>
+        <v>3.14658919228933</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.974799409038575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>